<commit_message>
Actualiza catálogos ISTAC/EUROSTAT y el dataset EDGAR (versión 2026)
Sincroniza ProyectoPersonal/SelecciónDatasetsProyecto tras regenerar los
catálogos de ISTAC y EUROSTAT (incluye la resolución de los topics
SIN_TOPIC_ASIGNAR en Eurostat.topics.xlsx) y reescribir EDGAR_GHG.Rmd para
el nuevo formato "booklet" que EDGAR publica desde 2026, con un fichero
nuevo (EDGAR_GHG_normalizado.rds) para las emisiones per cápita y por PIB.
</commit_message>
<xml_diff>
--- a/SelecciónDatasetsProyecto/EUROSTAT/Eurostat.topics.xlsx
+++ b/SelecciónDatasetsProyecto/EUROSTAT/Eurostat.topics.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="450">
   <si>
     <t xml:space="preserve">topic</t>
   </si>
@@ -1217,7 +1217,7 @@
     <t xml:space="preserve">SUPPLY_USE_IO_TABLES</t>
   </si>
   <si>
-    <t xml:space="preserve">Supply, use and input-output tables (SUIOTs) are matrices that provide a detailed picture of how goods and services are supplied and used in an economy. By balancing data from various sources in a consistent framework, they allow compiling a single coherent estimate of gross domestic product (GDP) based on production, expenditure, and income. SUIOTs comprise four main types of tables: Supply table: This table depicts how products (in rows) enter the economy, either through domestic production by industries or imports (in columns). The supply table also includes data on trade and transport margins as well as taxes less subsidies (in columns) to convert total supply from basic prices to purchasers' prices. Use table: This table depicts how products (in rows) are used by the economy, either for intermediate consumption by industries, or for final uses (both in columns). Final uses are disaggregated into 1) final consumption expenditure by households, general government, and non-profit institutions serving households, 2) gross capital formation and 3) exports. The use table contains additional rows to show, for each industry, how gross value added is generated, distinguishing compensation of employees, other taxes less subsidies on production, consumption of fixed capital, and net operating surplus and mixed income. The use table can refer to all transactions, domestic transactions or imported products. Input-output table: This table captures the supply and use of products in a single matrix, depicting either products or industries in both rows and columns. Similar to use tables, input-output tables can refer to all transactions, domestic transactions or imported products. Margin tables: These tables present separately 1) trade and transport margins and 2) taxes less subsidies, by products (in rows) and industries (in columns). The supply-use system is built upon two fundamental equations: total supply = production + imports = intermediate consumption + final consumption + gross capital formation + exports = total use (this equation is satisfied for any given product category) value added = production – intermediate consumption = compensation of employees + gross operating surplus and mixed income + other taxes less subsidies on production (this equation is satisfied for any given economic activity). SUIOTs distinguish 64 product and industry categories. Products are classified according to the statistical classification of products by activity (CPA 2.1). Industries are classified according to the statistical classification of economic activities (NACE Revision 2). The data are presented in million euro and million national currency. Eurostat collects and publishes SUIOTs for the 27 European Union (EU) countries, the countries of the European Free Trade Association (EFTA), and the EU enlargement countries. The tables are compiled in line with the European System of Accounts - ESA 2010 and the related transmission programme. Countries should deliver their SUIOTs 36 months after the end of the reference year according to the ESA 2010 transmission programme. This means that, for example, data for the year 2022 must be transmitted by 31 December 2025. SUIOTs comprise annual and 5-yearly data transmissions. The annual mandatory data transmission includes the supply table at basic prices, including transformation into purchasers' prices (T1500) and the use table in purchasers' prices (T1600), both in current and previous year’s prices. The 5-yearly mandatory data transmissions concerns years ending with ‘0’ or ‘5’ and includes the following tables: use table at basic prices (T1610) use table for domestic output at basic prices (T1611) use table for imports at basic prices (T1612) table of trade and transport margins (T1620) table of taxes less subsidies on products (T1630) symmetric input-output table at basic prices (T1700/50) symmetric input-output table for domestic output at basic prices (T1800/50) symmetric input-output table for imports at basic prices (T1900/50). The 5-yearly tables are to be transmitted in current prices. Countries are free to compile their input-output tables in product-by-product or industry-by-industry format. Eurostat encourages voluntary data transmissions. Several countries provide, e.g., 5-yearly tables on an annual basis or in both current and previous year’s prices. Eurostat publishes annual and 5-yearly tables in current prices from reference year 2010 onward and the annual tables in previous year’s prices from reference year 2015 onward. Next to publishing SUIOTs for individual countries, Eurostat compiles annually consolidated tables at current prices for the European Union (EU, that is, the 27 member countries as a whole) and the euro area (EA). The consolidated SUIOTs are based on the EU inter-country supply, use and input-output tables (EU inter-country SUIOTs; so-called FIGARO tables). Intra-EU and intra-EA trade are considered as domestic transactions. Imports and exports correspond to the respective trade in goods and services with countries outside of the European Union and the euro area, respectively. The regional breakdown of imports and exports in the SUIOTs for the EU and the EA is based on the country composition of both regions in the most recent reference year, and this composition is applied to the entire time series. This approach ensures consistency over time. However, it deviates from the approach used for the SUIOTs of individual countries, where an evolving country composition reflects the member countries of the EU and the EA in each respective year.</t>
+    <t xml:space="preserve">Supply, use and input-output tables (SUIOTs) are matrices that provide a detailed picture of how goods and services are supplied and used in an economy. By balancing data from various sources in a consistent framework, they allow compiling a single coherent estimate of gross domestic product (GDP) based on production, expenditure, and income. SUIOTs comprise four main types of tables: Supply table: This table depicts how products (in rows) enter the economy, either through domestic production by industries or imports (in columns). The supply table also includes data on trade and transport margins as well as taxes less subsidies (in columns) to convert total supply from basic prices to purchasers' prices. Use table: This table depicts how products (in rows) are used by the economy, either for intermediate consumption by industries, or for final uses (both in columns). Final uses are disaggregated into 1) final consumption expenditure by households, general government, and non-profit institutions serving households, 2) gross capital formation and 3) exports. The use table contains additional rows to show, for each industry, how gross value added is generated, distinguishing compensation of employees, other taxes less subsidies on production, consumption of fixed capital, and net operating surplus and mixed income. The use table can refer to all transactions, domestic transactions or imported products. Input-output table: This table captures the supply and use of products in a single matrix, depicting either products or industries in both rows and columns. Similar to use tables, input-output tables can refer to all transactions, domestic transactions or imported products. Margin tables: These tables present separately 1) trade and transport margins and 2) taxes less subsidies, by products (in rows) and industries and final uses (in columns). The supply-use system is built upon two fundamental equations: total supply = production + imports = intermediate consumption + final consumption + gross capital formation + exports = total use (this equation is satisfied for any given product category) value added = production – intermediate consumption = compensation of employees + gross operating surplus and mixed income + other taxes less subsidies on production (this equation is satisfied for any given economic activity). SUIOTs distinguish 64 product and industry categories. Products are classified according to the statistical classification of products by activity (CPA 2.1). Industries are classified according to the statistical classification of economic activities (NACE Revision 2). The data are presented in million euro and million national currency. Eurostat collects and publishes SUIOTs for the 27 European Union (EU) countries, the countries of the European Free Trade Association (EFTA), and the EU enlargement countries. The tables are compiled in line with the European System of Accounts - ESA 2010 and the related transmission programme. Countries should deliver their SUIOTs 36 months after the end of the reference year according to the ESA 2010 transmission programme. This means that, for example, data for the year 2022 must be transmitted by 31 December 2025. SUIOTs comprise annual and 5-yearly data transmissions. The annual mandatory data transmission includes the supply table at basic prices, including transformation into purchasers' prices (T1500) and the use table in purchasers' prices (T1600), both in current and previous year’s prices. The 5-yearly mandatory data transmissions concern years ending with ‘0’ or ‘5’ and include the following tables: use table at basic prices (T1610) use table for domestic output at basic prices (T1611) use table for imports at basic prices (T1612) table of trade and transport margins (T1620) table of taxes less subsidies on products (T1630) symmetric input-output table at basic prices (T1700/50) symmetric input-output table for domestic output at basic prices (T1800/50) symmetric input-output table for imports at basic prices (T1900/50). The 5-yearly tables are to be transmitted in current prices. Countries are free to compile their input-output tables in product-by-product or industry-by-industry format. Eurostat encourages voluntary data transmissions. Several countries provide, e.g., 5-yearly tables on an annual basis or in both current and previous year’s prices. Eurostat publishes annual and 5-yearly tables in current prices from reference year 2010 onward and the annual tables in previous year’s prices from reference year 2015 onward. Next to publishing SUIOTs for individual countries, Eurostat compiles annually consolidated tables at current prices for the European Union (EU, that is, the 27 member countries as a whole) and the euro area (EA). The consolidated SUIOTs are based on the EU inter-country supply, use and input-output tables (EU inter-country SUIOTs; so-called FIGARO tables). Intra-EU and intra-EA trade are considered as domestic transactions. Imports and exports correspond to the respective trade in goods and services with countries outside of the European Union and the euro area, respectively. The regional breakdown of imports and exports in the SUIOTs for the EU and the EA is based on the country composition of both regions in the most recent reference year, and this composition is applied to the entire time series. This approach ensures consistency over time. However, it deviates from the approach used for the SUIOTs of individual countries, where an evolving country composition reflects the member countries of the EU and the EA in each respective year.</t>
   </si>
   <si>
     <t xml:space="preserve">TEMPORARY_PROTECTION_DECISIONS</t>
@@ -1344,6 +1344,24 @@
   </si>
   <si>
     <t xml:space="preserve">The domain 'Youth Employment' is based on the results of the European Union Labour Force Survey (EU-LFS). The EU-LFS is a quarterly household sample survey carried out in the Member States of the European Union, EFTA countries (except for Liechtenstein) and Candidate Countries (Montenegro, North Macedonia, Serbia and Turkey). It is the main source of information about the situation and trends on the labour market in the European Union. Since 1 January 2021, the EU-LFS is based on Regulation (EU) 2019/1700, also called the Integrated European Social Statistics Framework Regulation (IESS FR), and its Commission Implementing Regulation (EU) 2019/2240. According to the regulations in force since 1 January 2021, the EU-LFS is organised in 9 topics: Technical items Person and household characteristics; Labour market participation; Educational attainment and background; Job tenure, work biography and previous work experience; Working conditions including working hours and working time arrangements; Participation in education and training; Health: status and disability, access to, availability and use of health care and health determinants; Income, consumption and elements of wealth, including debts. The survey's target population consists of all persons in private households, although the variables related to labour market are only collected for persons aged 15-89 years and education and training for persons aged 15-74 years. Detailed information on main features, legal basis, methodology and data as well as on the historical development of the EU-LFS is available on the EU-LFS (Statistics Explained) webpage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIR_POLLUTANTS_BY_SECTOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The European Union (EU) as a party to the Convention on Long-range Transboundary Air Pollution (LRTAP Convention) reports annually its air pollution inventory for the year t-2 and within the area covered by its Member States. Under the Convention, parties are obliged to report emissions data for numerous air pollutants. This dataset includes data on air pollutants: sulphur oxides (SOx), ammonia (NH3), nitrogen oxides (NOx), non-methane volatile organic compounds (NMVOCs), particulate matters (PM10, PM2.5), Lead (Pb), Cadmium (Cd), Mercury (Hg), Arsenic (As), Chromium (Cr) Copper (Cu), Nickel (Ni), Selenium (Se) and Zinc (Zn), as reported to the European Environment Agency (EEA). The EU inventory is fully consistent with national air pollution inventories compiled by the EU Member States. Note that Eurostat is not the producer of these data, only re-publishes them. The producer of the data is the European Environment Agency. Note that in the European Union emission inventory report 1990-2019 under the UNECE Convention on Long-range Transboundary Air Pollution, EU-28 totals do not include data from the United Kingdom. Therefore, Eurostat labels the same totals as EU-27.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PESTICIDE_USE_IN_AGRICULTURE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The data set comprises the quantity of each active substance contained in plant protection products used on a selected crop on an aggregated level from 2010 onwards. The data collection takes place every five years and the first reference year was 2010. According to Regulation (EC) No 1185/2009, the data collection is mandatory for all Member States of the European Union, Norway and Iceland, and optional for other EFTA countries as well as for candidate and potential candidate countries. The regulation stipulates that countries should collect data at least for one year out of the five-year period. Accordingly, some countries send data for one year only, others for more than one year, others for all five years, and some send even data on different crops in different years, because they have e.g. a vegetable survey in one year and a cereals survey in another year. The active substances are listed in Annex III of Regulation (EC) No 1185/2009 as amended by Commission Regulation (EU) 2017/269 of 16 February 2017. The quantity of active substances is expressed in kilograms. Eurostat disseminates the active substances on the three aggregation levels available in the harmonised classification of substances, called major groups (first level), categories of products (second level) and chemical classes (third level). The major groups are divided in the following categories: F – Fungicides and bactericides; H – Herbicides, haulm destructors and moss killers; I – Insecticides and acaricides; M – Molluscicides; PGR – Plant growth regulators; and ZR – Other plant protection products. The full code list of active substances and their aggregation levels is annexed at the end of this report (Annex name: 'List of active substances'). The disseminated data excludes micro-biological substances because of the difficulties to convert units used to express them (such as colony-forming unit (CFU)) into kilogram (kg), the reporting unit used for dissemination. The area treated with each substance is expressed in hectares. For the data between 2010-2014, the area treated cannot be disseminated, because the values are likely to contain double counting. That means if individual active substances of the same aggregation are applied on the same physical area, the area treated should not be added up not to double the area in the statistics reported. Only for Cyprus, the area treated could be published for 2011-2014, because they sent revisions in 2021 and can guarantee to have double counting excluded. For the five-year period 2015-2019, only the countries that ensured to have double-counting excluded were providing the information, and for these countries the hectare values were published. The selection of crops also differs widely between countries. The regulation stipulates that the crops selected by a country shall be representative of the crops cultivated in the Member State and of the substances used. This led e.g. to a variety of 174 crop codes used in total by all reporting countries for the first 5-year period 2010-2014, and 167 crop codes used in the second 5 years period 2015-2019. Considering all these different variables (164 aggregation levels of active substances, 5 reference years and about 200 crop codes free to choose), this results in a data set of more than 4 million possibilities for data combinations. The data set thus contains a lot of null values (a combination not available for a country).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PESTICIDE_HARMONISED_RISK_INDICATOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harmonised risk indicators are established in order to measure the progress achieved in meeting the objectives of the Directive 2009/128/EC on the sustainable use of pesticides. The data set shows the values of the Harmonised risk indicator 1 (HRI 1 - hereafter referred to as ‘the Harmonised risk indicator’), established in Commission Directive (EU) 2019/782 of 15 May 2019, amending Directive 2009/128/EC of the European Parliament and of the Council as regards the establishment of harmonised risk indicators. The indicator is presented as indices relative to a baseline of 100 (see section 3.9). The Harmonised risk indicator is based on statistics on the quantity of active substances in plant protection products placed on the market under Regulation (EC) No 1107/2009, provided to Eurostat according to Annex I of Regulation (EC) No 1185/2009. Those data are categorised into 4 risk groups and multiplied by hazard weightings established in Commission Directive (EU) 2019/782. The results of the calculations are then aggregated. The Member States and the Commission shall calculate and publish the Harmonised risk indicator in accordance with Articles 15(2) and 15(4) of Directive 2009/128/EC for each calendar year. The results of the calculations are available at the latest 20 months after the reference year. Eurostat calculates the EU-level indicator. Eurostat also calculates the national Harmonised risk indicator on behalf of Member States as a service. Member States make the information available to the public before 30 August each year.</t>
   </si>
 </sst>
 </file>
@@ -3448,6 +3466,30 @@
         <v>443</v>
       </c>
     </row>
+    <row r="223">
+      <c r="A223" t="s">
+        <v>444</v>
+      </c>
+      <c r="B223" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="s">
+        <v>446</v>
+      </c>
+      <c r="B224" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="s">
+        <v>448</v>
+      </c>
+      <c r="B225" t="s">
+        <v>449</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>